<commit_message>
update change notes and prepare release 0.1.0-ballot 0294e60d7baf764c8f03d6afb40b029a215b8289
</commit_message>
<xml_diff>
--- a/nr-prepare-release/ig/StructureDefinition-ActiviteEnseignement.xlsx
+++ b/nr-prepare-release/ig/StructureDefinition-ActiviteEnseignement.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>0.1.0-ballot</t>
   </si>
   <si>
     <t>Name</t>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-20T07:37:42+00:00</t>
+    <t>2026-04-20T08:03:20+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>